<commit_message>
test: suite pytest UNIT/INT con evidencia SENA
</commit_message>
<xml_diff>
--- a/docs/pruebas/Plan_de_Pruebas_PlomApp_SENA.xlsx
+++ b/docs/pruebas/Plan_de_Pruebas_PlomApp_SENA.xlsx
@@ -2453,7 +2453,7 @@
       </c>
       <c r="G8" s="62" t="inlineStr">
         <is>
-          <t>No ejecutado aún (fase de diseño).</t>
+          <t>Aprobado: 23/23 casos parametrizados (email, teléfono, contraseña, nombre y fecha/hora).</t>
         </is>
       </c>
       <c r="H8" s="61" t="inlineStr">
@@ -2463,7 +2463,7 @@
       </c>
       <c r="I8" s="61" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Exitoso</t>
         </is>
       </c>
       <c r="J8" s="61" t="inlineStr">
@@ -2473,12 +2473,12 @@
       </c>
       <c r="K8" s="63" t="inlineStr">
         <is>
-          <t>Planificado: api/tests/unit/test_validators.py</t>
+          <t>pytest -m unit: 35 passed; api/tests/unit/test_unit_01_validators.py</t>
         </is>
       </c>
       <c r="L8" s="62" t="inlineStr">
         <is>
-          <t>Cubre validación de entrada del registro; ejecutar con pytest -m unit.</t>
+          <t>Ejecutado el 26/10/2026 en SQLite en memoria; sin defectos.</t>
         </is>
       </c>
     </row>
@@ -2521,7 +2521,7 @@
       </c>
       <c r="G9" s="62" t="inlineStr">
         <is>
-          <t>No ejecutado aún (fase de diseño).</t>
+          <t>Aprobado: 4/4 casos (token válido con sub string, expiración, firma alterada y token inválido).</t>
         </is>
       </c>
       <c r="H9" s="61" t="inlineStr">
@@ -2531,7 +2531,7 @@
       </c>
       <c r="I9" s="61" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Exitoso</t>
         </is>
       </c>
       <c r="J9" s="61" t="inlineStr">
@@ -2541,12 +2541,12 @@
       </c>
       <c r="K9" s="63" t="inlineStr">
         <is>
-          <t>Planificado: api/tests/unit/test_jwt_utils.py</t>
+          <t>pytest -m unit: 35 passed; api/tests/unit/test_unit_02_jwt.py</t>
         </is>
       </c>
       <c r="L9" s="62" t="inlineStr">
         <is>
-          <t>Valida compatibilidad con tokens emitidos por Flask (sub string).</t>
+          <t>Ejecutado el 26/10/2026; se verificó compatibilidad HS256 con el contrato Flask.</t>
         </is>
       </c>
     </row>
@@ -2590,7 +2590,7 @@
       </c>
       <c r="G10" s="62" t="inlineStr">
         <is>
-          <t>No ejecutado aún (fase de diseño).</t>
+          <t>Aprobado: 3/3 pruebas (10 slots, conflicto 09:00, hoy sin slots pasados y transiciones de estado).</t>
         </is>
       </c>
       <c r="H10" s="61" t="inlineStr">
@@ -2600,7 +2600,7 @@
       </c>
       <c r="I10" s="61" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Exitoso</t>
         </is>
       </c>
       <c r="J10" s="61" t="inlineStr">
@@ -2610,12 +2610,12 @@
       </c>
       <c r="K10" s="63" t="inlineStr">
         <is>
-          <t>Planificado: api/tests/unit/test_appointment_slots.py</t>
+          <t>pytest -m unit: 35 passed; api/tests/unit/test_unit_03_appointment_slots.py</t>
         </is>
       </c>
       <c r="L10" s="62" t="inlineStr">
         <is>
-          <t>Sensible a zona horaria: fijar TZ y usar freezegun.</t>
+          <t>Ejecutado el 26/10/2026 con freezegun; sin defectos.</t>
         </is>
       </c>
     </row>
@@ -2658,7 +2658,7 @@
       </c>
       <c r="G11" s="62" t="inlineStr">
         <is>
-          <t>No ejecutado aún (fase de diseño).</t>
+          <t>Aprobado: 5/5 casos (parseo válido/inválido, coseno 1.0, 0.0 y casos límite).</t>
         </is>
       </c>
       <c r="H11" s="61" t="inlineStr">
@@ -2668,7 +2668,7 @@
       </c>
       <c r="I11" s="61" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Exitoso</t>
         </is>
       </c>
       <c r="J11" s="61" t="inlineStr">
@@ -2678,12 +2678,12 @@
       </c>
       <c r="K11" s="63" t="inlineStr">
         <is>
-          <t>Planificado: api/tests/unit/test_embedding_math.py</t>
+          <t>pytest -m unit: 35 passed; api/tests/unit/test_unit_04_embedding_math.py</t>
         </is>
       </c>
       <c r="L11" s="62" t="inlineStr">
         <is>
-          <t>No requiere pgvector; prueba la lógica de fallback en Python.</t>
+          <t>Ejecutado el 26/10/2026; no requiere pgvector ni red.</t>
         </is>
       </c>
     </row>
@@ -2726,7 +2726,7 @@
       </c>
       <c r="G12" s="62" t="inlineStr">
         <is>
-          <t>No ejecutado aún (fase de diseño).</t>
+          <t>Aprobado: 6/6 pruebas Vitest (email, nombre, teléfono, contraseña, registro y login).</t>
         </is>
       </c>
       <c r="H12" s="61" t="inlineStr">
@@ -2736,7 +2736,7 @@
       </c>
       <c r="I12" s="61" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Exitoso</t>
         </is>
       </c>
       <c r="J12" s="61" t="inlineStr">
@@ -2746,12 +2746,12 @@
       </c>
       <c r="K12" s="63" t="inlineStr">
         <is>
-          <t>Planificado: tests/unit/validation.test.js</t>
+          <t>npm run test:unit: 6 passed; tests/unit/unit_05_validation.test.js</t>
         </is>
       </c>
       <c r="L12" s="62" t="inlineStr">
         <is>
-          <t>Complementa la validación del backend; ejecutar con npm run test:unit.</t>
+          <t>Ejecutado el 26/10/2026 con Vitest 5.0.5 + jsdom 29.1.1.</t>
         </is>
       </c>
     </row>
@@ -4508,7 +4508,7 @@
       </c>
       <c r="G8" s="62" t="inlineStr">
         <is>
-          <t>10/10 tests del contrato OK (SQLite) el 26/10/2026: register 201, login 200, profile 401 sin token, password incorrecta 401.</t>
+          <t>Aprobado: 2/2 pruebas en PostgreSQL de pruebas (registro 201, login 200, perfil 200 y contraseña incorrecta 401).</t>
         </is>
       </c>
       <c r="H8" s="61" t="inlineStr">
@@ -4528,12 +4528,12 @@
       </c>
       <c r="K8" s="63" t="inlineStr">
         <is>
-          <t>manage.py test: 10/10 OK; api/tests/integration/test_auth_api.py (pendiente Postgres)</t>
+          <t>pytest -m integration --create-db (TEST_USE_CONFIGURED_DB=1): 8 passed; api/tests/integration/test_int_01_auth_api.py</t>
         </is>
       </c>
       <c r="L8" s="62" t="inlineStr">
         <is>
-          <t>Evidencia preliminar en SQLite; repetir en Postgres de pruebas antes de cerrar.</t>
+          <t>Ejecutado el 26/10/2026 contra test_plomapp en PostgreSQL 5434; la BD real no se modificó.</t>
         </is>
       </c>
     </row>
@@ -4574,7 +4574,7 @@
       </c>
       <c r="G9" s="62" t="inlineStr">
         <is>
-          <t>No ejecutado aún de forma automatizada; smoke 98/98 en clon y /api/appointments 200 como evidencia preliminar.</t>
+          <t>Aprobado: disponibilidad 200 con slot 09:00, creación 201, duplicado 409 y una sola cita persistida.</t>
         </is>
       </c>
       <c r="H9" s="61" t="inlineStr">
@@ -4584,7 +4584,7 @@
       </c>
       <c r="I9" s="61" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Exitoso</t>
         </is>
       </c>
       <c r="J9" s="61" t="inlineStr">
@@ -4594,12 +4594,12 @@
       </c>
       <c r="K9" s="63" t="inlineStr">
         <is>
-          <t>Planificado: api/tests/integration/test_appointments_api.py; smoke 98/98 (clon)</t>
+          <t>pytest -m integration --create-db (TEST_USE_CONFIGURED_DB=1): 8 passed; api/tests/integration/test_int_02_appointments_api.py</t>
         </is>
       </c>
       <c r="L9" s="62" t="inlineStr">
         <is>
-          <t>Requiere PostgreSQL: select_for_update no aplica en SQLite.</t>
+          <t>Ejecutado en PostgreSQL de pruebas; valida select_for_update y la regla de no doble reserva.</t>
         </is>
       </c>
     </row>
@@ -4640,7 +4640,7 @@
       </c>
       <c r="G10" s="62" t="inlineStr">
         <is>
-          <t>No ejecutado aún de forma automatizada; verificación manual: vector 0.8.6, HNSW, similitud 1.0 y búsqueda con resultados.</t>
+          <t>Aprobado: sincronización de 1 servicio, columna vector(512), índice HNSW y búsqueda con similitud 1.0.</t>
         </is>
       </c>
       <c r="H10" s="61" t="inlineStr">
@@ -4650,7 +4650,7 @@
       </c>
       <c r="I10" s="61" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Exitoso</t>
         </is>
       </c>
       <c r="J10" s="61" t="inlineStr">
@@ -4660,12 +4660,12 @@
       </c>
       <c r="K10" s="63" t="inlineStr">
         <is>
-          <t>Planificado: api/tests/integration/test_pgvector.py; verify_pgvector.py (manual)</t>
+          <t>pytest -m integration --create-db (TEST_USE_CONFIGURED_DB=1): 8 passed; api/tests/integration/test_int_03_pgvector.py</t>
         </is>
       </c>
       <c r="L10" s="62" t="inlineStr">
         <is>
-          <t>Mockear Voyage/Gemini para que la prueba sea determinista y no dependa de red.</t>
+          <t>Proveedor de embeddings mockeado; no se llamó a Voyage/Gemini. Extensión e índice creados en la BD de pruebas.</t>
         </is>
       </c>
     </row>
@@ -4708,7 +4708,7 @@
       </c>
       <c r="G11" s="62" t="inlineStr">
         <is>
-          <t>3/3 tests de upload OK el 26/10/2026 (PNG 201, falso 400, 11 MB 400); JSONB verificado en la BD real.</t>
+          <t>Aprobado: 4/4 pruebas (PNG 201, contenido falso 400, archivo &gt;10 MB 400 y evidence_photos JSONB/lista).</t>
         </is>
       </c>
       <c r="H11" s="61" t="inlineStr">
@@ -4728,12 +4728,12 @@
       </c>
       <c r="K11" s="62" t="inlineStr">
         <is>
-          <t>manage.py test: 3/3 upload OK; api/tests/integration/test_uploads_jsonb.py (planificado)</t>
+          <t>pytest -m integration --create-db (TEST_USE_CONFIGURED_DB=1): 8 passed; api/tests/integration/test_int_04_uploads_jsonb.py</t>
         </is>
       </c>
       <c r="L11" s="62" t="inlineStr">
         <is>
-          <t>Evitar escribir en static/uploads real; usar tmp_path/override_settings.</t>
+          <t>Uploads en tmp_path; JSONB verificado con information_schema en PostgreSQL de pruebas.</t>
         </is>
       </c>
     </row>
@@ -6406,7 +6406,7 @@
       </c>
       <c r="G8" s="62" t="inlineStr">
         <is>
-          <t>No ejecutado aún (fase de diseño).</t>
+          <t>No ejecutado: spec Playwright de login/dashboard creado; flujo completo de agendamiento pendiente de BD e2e, servidores y credenciales.</t>
         </is>
       </c>
       <c r="H8" s="61" t="inlineStr">
@@ -6426,12 +6426,12 @@
       </c>
       <c r="K8" s="63" t="inlineStr">
         <is>
-          <t>Planificado: e2e/tests/client.spec.js (Playwright + trace/video)</t>
+          <t>e2e/tests/e2e_01_client.spec.js (Playwright); npm run test:e2e</t>
         </is>
       </c>
       <c r="L8" s="62" t="inlineStr">
         <is>
-          <t>Agregar data-testid a login, agendar y tarjeta de cita; manejar alert() de sesión.</t>
+          <t>No se marca exitoso ni se inventan evidencias. El flujo completo requiere sembrar cliente, servicio y cita en una BD e2e.</t>
         </is>
       </c>
     </row>
@@ -6474,7 +6474,7 @@
       </c>
       <c r="G9" s="62" t="inlineStr">
         <is>
-          <t>No ejecutado aún (fase de diseño).</t>
+          <t>No ejecutado: spec Playwright de login/agenda creado; cambio de estado pendiente de BD e2e, servidores y credenciales.</t>
         </is>
       </c>
       <c r="H9" s="61" t="inlineStr">
@@ -6494,12 +6494,12 @@
       </c>
       <c r="K9" s="63" t="inlineStr">
         <is>
-          <t>Planificado: e2e/tests/technician.spec.js</t>
+          <t>e2e/tests/e2e_02_technician.spec.js (Playwright); npm run test:e2e</t>
         </is>
       </c>
       <c r="L9" s="62" t="inlineStr">
         <is>
-          <t>Validar que no se permita completed-&gt;scheduled; usar datos sembrados deterministas.</t>
+          <t>No se marca exitoso ni se inventan evidencias. Requiere cita asignada y transiciones sembradas.</t>
         </is>
       </c>
     </row>
@@ -6542,7 +6542,7 @@
       </c>
       <c r="G10" s="62" t="inlineStr">
         <is>
-          <t>No ejecutado aún (fase de diseño).</t>
+          <t>No ejecutado: spec Playwright de login/panel creado; gestión de cita pendiente de BD e2e, servidores y credenciales.</t>
         </is>
       </c>
       <c r="H10" s="61" t="inlineStr">
@@ -6562,12 +6562,12 @@
       </c>
       <c r="K10" s="63" t="inlineStr">
         <is>
-          <t>Planificado: e2e/tests/admin.spec.js</t>
+          <t>e2e/tests/e2e_03_admin.spec.js (Playwright); npm run test:e2e</t>
         </is>
       </c>
       <c r="L10" s="62" t="inlineStr">
         <is>
-          <t>Usar un admin de pruebas; no ejecutar contra la BD real.</t>
+          <t>No se marca exitoso ni se inventan evidencias. Usar un admin de pruebas, nunca la BD real.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: agrega 10 pruebas unitarias basicas y evidencia Excel
</commit_message>
<xml_diff>
--- a/docs/pruebas/Plan_de_Pruebas_PlomApp_SENA.xlsx
+++ b/docs/pruebas/Plan_de_Pruebas_PlomApp_SENA.xlsx
@@ -8,8 +8,11 @@
     <sheet name="Pruebas Integracion" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Pruebas E2E" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Guía del Aprendiz" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Unitarias Basicas" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Unitarias Basicas'!$A$7:$L$17</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -19,7 +22,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="19">
     <font>
       <name val="Calibri"/>
       <color theme="1"/>
@@ -79,8 +82,52 @@
       <color theme="1"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="001F2937"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00006100"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="006B7280"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="006B7280"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -117,8 +164,38 @@
         <bgColor rgb="FFF9FAFB"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000B4F26"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F3F4F6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00374151"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F9FAFB"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="22">
+  <borders count="23">
     <border/>
     <border>
       <left/>
@@ -253,11 +330,25 @@
         <color rgb="FFD1D5DB"/>
       </right>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D1D5DB"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D1D5DB"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D1D5DB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D1D5DB"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="78">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -400,6 +491,45 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="12" fillId="0" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="12" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="12" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -717,7 +847,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J25"/>
+  <dimension ref="A1:J26"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="18" customWidth="1" style="45" min="1" max="2"/>
@@ -1221,7 +1351,13 @@
       <c r="I25" s="22" t="n"/>
       <c r="J25" s="48" t="n"/>
     </row>
-    <row r="26" ht="15.75" customHeight="1" s="45"/>
+    <row r="26" ht="15.75" customHeight="1" s="45">
+      <c r="A26" s="65" t="inlineStr">
+        <is>
+          <t>ANEXO: la hoja 'Unitarias Basicas' contiene 10 pruebas unitarias básicas adicionales (UNIT-B01 a UNIT-B10) para la entrega del aprendiz.</t>
+        </is>
+      </c>
+    </row>
     <row r="27" ht="15.75" customHeight="1" s="45"/>
     <row r="28" ht="15.75" customHeight="1" s="45"/>
     <row r="29" ht="15.75" customHeight="1" s="45"/>
@@ -2197,7 +2333,7 @@
     <row r="999" ht="15.75" customHeight="1" s="45"/>
     <row r="1000" ht="15.75" customHeight="1" s="45"/>
   </sheetData>
-  <mergeCells count="44">
+  <mergeCells count="45">
     <mergeCell ref="F4:G4"/>
     <mergeCell ref="A12:B13"/>
     <mergeCell ref="A1:J2"/>
@@ -2240,6 +2376,7 @@
     <mergeCell ref="A19:B19"/>
     <mergeCell ref="H4:J4"/>
     <mergeCell ref="C4:E4"/>
+    <mergeCell ref="A26:J26"/>
     <mergeCell ref="F24:H24"/>
     <mergeCell ref="H6:J6"/>
   </mergeCells>
@@ -9223,4 +9360,793 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" style="45" min="1" max="1"/>
+    <col width="34" customWidth="1" style="45" min="2" max="2"/>
+    <col width="32" customWidth="1" style="45" min="3" max="3"/>
+    <col width="36" customWidth="1" style="45" min="4" max="4"/>
+    <col width="40" customWidth="1" style="45" min="5" max="5"/>
+    <col width="40" customWidth="1" style="45" min="6" max="6"/>
+    <col width="36" customWidth="1" style="45" min="7" max="7"/>
+    <col width="24" customWidth="1" style="45" min="8" max="8"/>
+    <col width="12" customWidth="1" style="45" min="9" max="9"/>
+    <col width="11" customWidth="1" style="45" min="10" max="10"/>
+    <col width="42" customWidth="1" style="45" min="11" max="11"/>
+    <col width="34" customWidth="1" style="45" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1" s="45">
+      <c r="A1" s="66" t="inlineStr">
+        <is>
+          <t>SENA - SIGA | ANEXO: 10 PRUEBAS UNITARIAS BÁSICAS (ENTREGA DEL APRENDIZ)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="67" t="inlineStr">
+        <is>
+          <t>Nivel de Prueba:</t>
+        </is>
+      </c>
+      <c r="C3" s="68" t="inlineStr">
+        <is>
+          <t>Nivel 1: Pruebas Unitarias (Unit Testing) - validadores puros</t>
+        </is>
+      </c>
+      <c r="G3" s="67" t="inlineStr">
+        <is>
+          <t>Enfoque:</t>
+        </is>
+      </c>
+      <c r="I3" s="68" t="inlineStr">
+        <is>
+          <t>Funciones de api/utils/validators.py; sin base de datos, servidor ni internet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="67" t="inlineStr">
+        <is>
+          <t>Total Ejecutadas:</t>
+        </is>
+      </c>
+      <c r="B5" s="69" t="n">
+        <v>10</v>
+      </c>
+      <c r="C5" s="67" t="inlineStr">
+        <is>
+          <t>Exitosas (Aprobadas):</t>
+        </is>
+      </c>
+      <c r="D5" s="69" t="n">
+        <v>10</v>
+      </c>
+      <c r="E5" s="67" t="inlineStr">
+        <is>
+          <t>Fallidas (Defectos):</t>
+        </is>
+      </c>
+      <c r="F5" s="69" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="67" t="inlineStr">
+        <is>
+          <t>Tasa de Éxito:</t>
+        </is>
+      </c>
+      <c r="H5" s="70" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" ht="44" customHeight="1" s="45">
+      <c r="A7" s="71" t="inlineStr">
+        <is>
+          <t>ID Caso</t>
+        </is>
+      </c>
+      <c r="B7" s="71" t="inlineStr">
+        <is>
+          <t>Componente / Escenario Probado</t>
+        </is>
+      </c>
+      <c r="C7" s="71" t="inlineStr">
+        <is>
+          <t>Precondiciones / Configuración</t>
+        </is>
+      </c>
+      <c r="D7" s="71" t="inlineStr">
+        <is>
+          <t>Datos de Entrada (Arrange)</t>
+        </is>
+      </c>
+      <c r="E7" s="71" t="inlineStr">
+        <is>
+          <t>Pasos de Ejecución (Act)</t>
+        </is>
+      </c>
+      <c r="F7" s="71" t="inlineStr">
+        <is>
+          <t>Resultado Esperado (Assert / Oráculo)</t>
+        </is>
+      </c>
+      <c r="G7" s="71" t="inlineStr">
+        <is>
+          <t>Resultado Obtenido en Ejecución</t>
+        </is>
+      </c>
+      <c r="H7" s="71" t="inlineStr">
+        <is>
+          <t>Tipo / Técnica</t>
+        </is>
+      </c>
+      <c r="I7" s="71" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="J7" s="71" t="inlineStr">
+        <is>
+          <t>Severidad / Prioridad</t>
+        </is>
+      </c>
+      <c r="K7" s="71" t="inlineStr">
+        <is>
+          <t>Evidencia (URL / Test Pass / Log)</t>
+        </is>
+      </c>
+      <c r="L7" s="71" t="inlineStr">
+        <is>
+          <t>Observaciones / Defecto Asociado</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="58" customHeight="1" s="45">
+      <c r="A8" s="72" t="inlineStr">
+        <is>
+          <t>UNIT-B01</t>
+        </is>
+      </c>
+      <c r="B8" s="73" t="inlineStr">
+        <is>
+          <t>Validación de email: caso válido</t>
+        </is>
+      </c>
+      <c r="C8" s="73" t="inlineStr">
+        <is>
+          <t>Función validate_email importada; sin BD ni servidor.</t>
+        </is>
+      </c>
+      <c r="D8" s="73" t="inlineStr">
+        <is>
+          <t>email="usuario@plomaap.com"</t>
+        </is>
+      </c>
+      <c r="E8" s="73" t="inlineStr">
+        <is>
+          <t>1. Llamar validate_email(email). / 2. Capturar el valor booleano.</t>
+        </is>
+      </c>
+      <c r="F8" s="73" t="inlineStr">
+        <is>
+          <t>Retorna True.</t>
+        </is>
+      </c>
+      <c r="G8" s="73" t="inlineStr">
+        <is>
+          <t>Aprobado: retornó True.</t>
+        </is>
+      </c>
+      <c r="H8" s="73" t="inlineStr">
+        <is>
+          <t>Caja Blanca (Partición equivalente)</t>
+        </is>
+      </c>
+      <c r="I8" s="74" t="inlineStr">
+        <is>
+          <t>Exitoso</t>
+        </is>
+      </c>
+      <c r="J8" s="72" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="K8" s="73" t="inlineStr">
+        <is>
+          <t>pytest api\tests\unit\test_unit_10_basicas.py -v: 10 passed; test_01_email_valido</t>
+        </is>
+      </c>
+      <c r="L8" s="73" t="inlineStr">
+        <is>
+          <t>Sin defectos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="58" customHeight="1" s="45">
+      <c r="A9" s="75" t="inlineStr">
+        <is>
+          <t>UNIT-B02</t>
+        </is>
+      </c>
+      <c r="B9" s="76" t="inlineStr">
+        <is>
+          <t>Validación de email: caso inválido</t>
+        </is>
+      </c>
+      <c r="C9" s="76" t="inlineStr">
+        <is>
+          <t>Función validate_email importada; sin BD ni servidor.</t>
+        </is>
+      </c>
+      <c r="D9" s="76" t="inlineStr">
+        <is>
+          <t>email="usuario@"</t>
+        </is>
+      </c>
+      <c r="E9" s="76" t="inlineStr">
+        <is>
+          <t>1. Llamar validate_email(email). / 2. Capturar el valor booleano.</t>
+        </is>
+      </c>
+      <c r="F9" s="76" t="inlineStr">
+        <is>
+          <t>Retorna False.</t>
+        </is>
+      </c>
+      <c r="G9" s="76" t="inlineStr">
+        <is>
+          <t>Aprobado: retornó False.</t>
+        </is>
+      </c>
+      <c r="H9" s="76" t="inlineStr">
+        <is>
+          <t>Caja Blanca (Partición equivalente)</t>
+        </is>
+      </c>
+      <c r="I9" s="74" t="inlineStr">
+        <is>
+          <t>Exitoso</t>
+        </is>
+      </c>
+      <c r="J9" s="75" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="K9" s="76" t="inlineStr">
+        <is>
+          <t>pytest api\tests\unit\test_unit_10_basicas.py -v: 10 passed; test_02_email_invalido</t>
+        </is>
+      </c>
+      <c r="L9" s="76" t="inlineStr">
+        <is>
+          <t>Sin defectos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="58" customHeight="1" s="45">
+      <c r="A10" s="72" t="inlineStr">
+        <is>
+          <t>UNIT-B03</t>
+        </is>
+      </c>
+      <c r="B10" s="73" t="inlineStr">
+        <is>
+          <t>Validación de teléfono: caso válido</t>
+        </is>
+      </c>
+      <c r="C10" s="73" t="inlineStr">
+        <is>
+          <t>Función validate_phone importada; sin BD ni servidor.</t>
+        </is>
+      </c>
+      <c r="D10" s="73" t="inlineStr">
+        <is>
+          <t>telefono="3229874810"</t>
+        </is>
+      </c>
+      <c r="E10" s="73" t="inlineStr">
+        <is>
+          <t>1. Llamar validate_phone(telefono). / 2. Capturar el valor booleano.</t>
+        </is>
+      </c>
+      <c r="F10" s="73" t="inlineStr">
+        <is>
+          <t>Retorna True.</t>
+        </is>
+      </c>
+      <c r="G10" s="73" t="inlineStr">
+        <is>
+          <t>Aprobado: retornó True.</t>
+        </is>
+      </c>
+      <c r="H10" s="73" t="inlineStr">
+        <is>
+          <t>Caja Blanca (Partición equivalente)</t>
+        </is>
+      </c>
+      <c r="I10" s="74" t="inlineStr">
+        <is>
+          <t>Exitoso</t>
+        </is>
+      </c>
+      <c r="J10" s="72" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="K10" s="73" t="inlineStr">
+        <is>
+          <t>pytest api\tests\unit\test_unit_10_basicas.py -v: 10 passed; test_03_telefono_valido</t>
+        </is>
+      </c>
+      <c r="L10" s="73" t="inlineStr">
+        <is>
+          <t>Sin defectos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="58" customHeight="1" s="45">
+      <c r="A11" s="75" t="inlineStr">
+        <is>
+          <t>UNIT-B04</t>
+        </is>
+      </c>
+      <c r="B11" s="76" t="inlineStr">
+        <is>
+          <t>Validación de teléfono: caso inválido</t>
+        </is>
+      </c>
+      <c r="C11" s="76" t="inlineStr">
+        <is>
+          <t>Función validate_phone importada; sin BD ni servidor.</t>
+        </is>
+      </c>
+      <c r="D11" s="76" t="inlineStr">
+        <is>
+          <t>telefono="123"</t>
+        </is>
+      </c>
+      <c r="E11" s="76" t="inlineStr">
+        <is>
+          <t>1. Llamar validate_phone(telefono). / 2. Capturar el valor booleano.</t>
+        </is>
+      </c>
+      <c r="F11" s="76" t="inlineStr">
+        <is>
+          <t>Retorna False.</t>
+        </is>
+      </c>
+      <c r="G11" s="76" t="inlineStr">
+        <is>
+          <t>Aprobado: retornó False.</t>
+        </is>
+      </c>
+      <c r="H11" s="76" t="inlineStr">
+        <is>
+          <t>Caja Blanca (Partición equivalente)</t>
+        </is>
+      </c>
+      <c r="I11" s="74" t="inlineStr">
+        <is>
+          <t>Exitoso</t>
+        </is>
+      </c>
+      <c r="J11" s="75" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="K11" s="76" t="inlineStr">
+        <is>
+          <t>pytest api\tests\unit\test_unit_10_basicas.py -v: 10 passed; test_04_telefono_invalido</t>
+        </is>
+      </c>
+      <c r="L11" s="76" t="inlineStr">
+        <is>
+          <t>Sin defectos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="58" customHeight="1" s="45">
+      <c r="A12" s="72" t="inlineStr">
+        <is>
+          <t>UNIT-B05</t>
+        </is>
+      </c>
+      <c r="B12" s="73" t="inlineStr">
+        <is>
+          <t>Validación de contraseña: caso válido</t>
+        </is>
+      </c>
+      <c r="C12" s="73" t="inlineStr">
+        <is>
+          <t>Función validate_password importada; sin BD ni servidor.</t>
+        </is>
+      </c>
+      <c r="D12" s="73" t="inlineStr">
+        <is>
+          <t>password="PlomApp2026*"</t>
+        </is>
+      </c>
+      <c r="E12" s="73" t="inlineStr">
+        <is>
+          <t>1. Llamar validate_password(password). / 2. Capturar el valor booleano.</t>
+        </is>
+      </c>
+      <c r="F12" s="73" t="inlineStr">
+        <is>
+          <t>Retorna True (8 caracteres o más).</t>
+        </is>
+      </c>
+      <c r="G12" s="73" t="inlineStr">
+        <is>
+          <t>Aprobado: retornó True.</t>
+        </is>
+      </c>
+      <c r="H12" s="73" t="inlineStr">
+        <is>
+          <t>Caja Blanca (Valor límite / partición)</t>
+        </is>
+      </c>
+      <c r="I12" s="74" t="inlineStr">
+        <is>
+          <t>Exitoso</t>
+        </is>
+      </c>
+      <c r="J12" s="72" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="K12" s="73" t="inlineStr">
+        <is>
+          <t>pytest api\tests\unit\test_unit_10_basicas.py -v: 10 passed; test_05_password_valido</t>
+        </is>
+      </c>
+      <c r="L12" s="73" t="inlineStr">
+        <is>
+          <t>Sin defectos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="58" customHeight="1" s="45">
+      <c r="A13" s="75" t="inlineStr">
+        <is>
+          <t>UNIT-B06</t>
+        </is>
+      </c>
+      <c r="B13" s="76" t="inlineStr">
+        <is>
+          <t>Validación de contraseña: caso corto</t>
+        </is>
+      </c>
+      <c r="C13" s="76" t="inlineStr">
+        <is>
+          <t>Función validate_password importada; sin BD ni servidor.</t>
+        </is>
+      </c>
+      <c r="D13" s="76" t="inlineStr">
+        <is>
+          <t>password="1234567"</t>
+        </is>
+      </c>
+      <c r="E13" s="76" t="inlineStr">
+        <is>
+          <t>1. Llamar validate_password(password). / 2. Capturar el valor booleano.</t>
+        </is>
+      </c>
+      <c r="F13" s="76" t="inlineStr">
+        <is>
+          <t>Retorna False (7 caracteres).</t>
+        </is>
+      </c>
+      <c r="G13" s="76" t="inlineStr">
+        <is>
+          <t>Aprobado: retornó False.</t>
+        </is>
+      </c>
+      <c r="H13" s="76" t="inlineStr">
+        <is>
+          <t>Caja Blanca (Valor límite / partición)</t>
+        </is>
+      </c>
+      <c r="I13" s="74" t="inlineStr">
+        <is>
+          <t>Exitoso</t>
+        </is>
+      </c>
+      <c r="J13" s="75" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="K13" s="76" t="inlineStr">
+        <is>
+          <t>pytest api\tests\unit\test_unit_10_basicas.py -v: 10 passed; test_06_password_corto</t>
+        </is>
+      </c>
+      <c r="L13" s="76" t="inlineStr">
+        <is>
+          <t>Sin defectos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="58" customHeight="1" s="45">
+      <c r="A14" s="72" t="inlineStr">
+        <is>
+          <t>UNIT-B07</t>
+        </is>
+      </c>
+      <c r="B14" s="73" t="inlineStr">
+        <is>
+          <t>Validación de nombre: caso válido</t>
+        </is>
+      </c>
+      <c r="C14" s="73" t="inlineStr">
+        <is>
+          <t>Función validate_name importada; sin BD ni servidor.</t>
+        </is>
+      </c>
+      <c r="D14" s="73" t="inlineStr">
+        <is>
+          <t>nombre="Andrés"</t>
+        </is>
+      </c>
+      <c r="E14" s="73" t="inlineStr">
+        <is>
+          <t>1. Llamar validate_name(nombre). / 2. Capturar el valor booleano.</t>
+        </is>
+      </c>
+      <c r="F14" s="73" t="inlineStr">
+        <is>
+          <t>Retorna True (2 caracteres o más).</t>
+        </is>
+      </c>
+      <c r="G14" s="73" t="inlineStr">
+        <is>
+          <t>Aprobado: retornó True.</t>
+        </is>
+      </c>
+      <c r="H14" s="73" t="inlineStr">
+        <is>
+          <t>Caja Blanca (Partición equivalente)</t>
+        </is>
+      </c>
+      <c r="I14" s="74" t="inlineStr">
+        <is>
+          <t>Exitoso</t>
+        </is>
+      </c>
+      <c r="J14" s="72" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="K14" s="73" t="inlineStr">
+        <is>
+          <t>pytest api\tests\unit\test_unit_10_basicas.py -v: 10 passed; test_07_nombre_valido</t>
+        </is>
+      </c>
+      <c r="L14" s="73" t="inlineStr">
+        <is>
+          <t>Sin defectos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="58" customHeight="1" s="45">
+      <c r="A15" s="75" t="inlineStr">
+        <is>
+          <t>UNIT-B08</t>
+        </is>
+      </c>
+      <c r="B15" s="76" t="inlineStr">
+        <is>
+          <t>Validación de nombre: caso corto</t>
+        </is>
+      </c>
+      <c r="C15" s="76" t="inlineStr">
+        <is>
+          <t>Función validate_name importada; sin BD ni servidor.</t>
+        </is>
+      </c>
+      <c r="D15" s="76" t="inlineStr">
+        <is>
+          <t>nombre="A"</t>
+        </is>
+      </c>
+      <c r="E15" s="76" t="inlineStr">
+        <is>
+          <t>1. Llamar validate_name(nombre). / 2. Capturar el valor booleano.</t>
+        </is>
+      </c>
+      <c r="F15" s="76" t="inlineStr">
+        <is>
+          <t>Retorna False (1 carácter).</t>
+        </is>
+      </c>
+      <c r="G15" s="76" t="inlineStr">
+        <is>
+          <t>Aprobado: retornó False.</t>
+        </is>
+      </c>
+      <c r="H15" s="76" t="inlineStr">
+        <is>
+          <t>Caja Blanca (Valor límite / partición)</t>
+        </is>
+      </c>
+      <c r="I15" s="74" t="inlineStr">
+        <is>
+          <t>Exitoso</t>
+        </is>
+      </c>
+      <c r="J15" s="75" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="K15" s="76" t="inlineStr">
+        <is>
+          <t>pytest api\tests\unit\test_unit_10_basicas.py -v: 10 passed; test_08_nombre_corto</t>
+        </is>
+      </c>
+      <c r="L15" s="76" t="inlineStr">
+        <is>
+          <t>Sin defectos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="58" customHeight="1" s="45">
+      <c r="A16" s="72" t="inlineStr">
+        <is>
+          <t>UNIT-B09</t>
+        </is>
+      </c>
+      <c r="B16" s="73" t="inlineStr">
+        <is>
+          <t>Validación de fecha y hora: caso válido</t>
+        </is>
+      </c>
+      <c r="C16" s="73" t="inlineStr">
+        <is>
+          <t>Función validate_date_time importada; sin BD ni servidor.</t>
+        </is>
+      </c>
+      <c r="D16" s="73" t="inlineStr">
+        <is>
+          <t>fecha="2026-11-02" / hora="09:00"</t>
+        </is>
+      </c>
+      <c r="E16" s="73" t="inlineStr">
+        <is>
+          <t>1. Llamar validate_date_time(fecha, hora). / 2. Capturar el valor booleano.</t>
+        </is>
+      </c>
+      <c r="F16" s="73" t="inlineStr">
+        <is>
+          <t>Retorna True.</t>
+        </is>
+      </c>
+      <c r="G16" s="73" t="inlineStr">
+        <is>
+          <t>Aprobado: retornó True.</t>
+        </is>
+      </c>
+      <c r="H16" s="73" t="inlineStr">
+        <is>
+          <t>Caja Blanca (Formato / partición)</t>
+        </is>
+      </c>
+      <c r="I16" s="74" t="inlineStr">
+        <is>
+          <t>Exitoso</t>
+        </is>
+      </c>
+      <c r="J16" s="72" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="K16" s="73" t="inlineStr">
+        <is>
+          <t>pytest api\tests\unit\test_unit_10_basicas.py -v: 10 passed; test_09_fecha_y_hora_validas</t>
+        </is>
+      </c>
+      <c r="L16" s="73" t="inlineStr">
+        <is>
+          <t>Sin defectos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="58" customHeight="1" s="45">
+      <c r="A17" s="75" t="inlineStr">
+        <is>
+          <t>UNIT-B10</t>
+        </is>
+      </c>
+      <c r="B17" s="76" t="inlineStr">
+        <is>
+          <t>Validación de fecha y hora: caso inválido</t>
+        </is>
+      </c>
+      <c r="C17" s="76" t="inlineStr">
+        <is>
+          <t>Función validate_date_time importada; sin BD ni servidor.</t>
+        </is>
+      </c>
+      <c r="D17" s="76" t="inlineStr">
+        <is>
+          <t>fecha="2026-13-01" / hora="09:00"</t>
+        </is>
+      </c>
+      <c r="E17" s="76" t="inlineStr">
+        <is>
+          <t>1. Llamar validate_date_time(fecha, hora). / 2. Capturar el valor booleano.</t>
+        </is>
+      </c>
+      <c r="F17" s="76" t="inlineStr">
+        <is>
+          <t>Retorna False (mes 13 inexistente).</t>
+        </is>
+      </c>
+      <c r="G17" s="76" t="inlineStr">
+        <is>
+          <t>Aprobado: retornó False.</t>
+        </is>
+      </c>
+      <c r="H17" s="76" t="inlineStr">
+        <is>
+          <t>Caja Blanca (Valor inválido / formato)</t>
+        </is>
+      </c>
+      <c r="I17" s="74" t="inlineStr">
+        <is>
+          <t>Exitoso</t>
+        </is>
+      </c>
+      <c r="J17" s="75" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="K17" s="76" t="inlineStr">
+        <is>
+          <t>pytest api\tests\unit\test_unit_10_basicas.py -v: 10 passed; test_10_fecha_y_hora_invalidas</t>
+        </is>
+      </c>
+      <c r="L17" s="76" t="inlineStr">
+        <is>
+          <t>Sin defectos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="34" customHeight="1" s="45">
+      <c r="A19" s="77" t="inlineStr">
+        <is>
+          <t>NOTA: estas 10 pruebas unitarias básicas son un anexo de la entrega del aprendiz. No reemplazan los casos UNIT-01 a UNIT-05 del plan SENA ni modifican el resumen general de 12 casos.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A7:L17"/>
+  <mergeCells count="6">
+    <mergeCell ref="C3:F3"/>
+    <mergeCell ref="A19:L19"/>
+    <mergeCell ref="I3:L3"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="G3:H3"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fix: reemplaza casos unitarios del Excel por las 10 pruebas basicas
</commit_message>
<xml_diff>
--- a/docs/pruebas/Plan_de_Pruebas_PlomApp_SENA.xlsx
+++ b/docs/pruebas/Plan_de_Pruebas_PlomApp_SENA.xlsx
@@ -8,11 +8,8 @@
     <sheet name="Pruebas Integracion" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Pruebas E2E" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Guía del Aprendiz" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Unitarias Basicas" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Unitarias Basicas'!$A$7:$L$17</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -22,7 +19,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="19">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <color theme="1"/>
@@ -82,52 +79,8 @@
       <color theme="1"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="13"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="001F2937"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00006100"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <i val="1"/>
-      <color rgb="006B7280"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <i val="1"/>
-      <color rgb="006B7280"/>
-      <sz val="9"/>
-    </font>
   </fonts>
-  <fills count="13">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -164,38 +117,8 @@
         <bgColor rgb="FFF9FAFB"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="000B4F26"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F3F4F6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00374151"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F9FAFB"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="23">
+  <borders count="22">
     <border/>
     <border>
       <left/>
@@ -330,25 +253,11 @@
         <color rgb="FFD1D5DB"/>
       </right>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="00D1D5DB"/>
-      </left>
-      <right style="thin">
-        <color rgb="00D1D5DB"/>
-      </right>
-      <top style="thin">
-        <color rgb="00D1D5DB"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00D1D5DB"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="78">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -492,44 +401,8 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="9" fontId="3" fillId="4" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="12" fillId="0" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="9" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="10" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="10" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="11" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="12" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="12" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -847,7 +720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J26"/>
+  <dimension ref="A1:J25"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="18" customWidth="1" style="45" min="1" max="2"/>
@@ -1351,13 +1224,7 @@
       <c r="I25" s="22" t="n"/>
       <c r="J25" s="48" t="n"/>
     </row>
-    <row r="26" ht="15.75" customHeight="1" s="45">
-      <c r="A26" s="65" t="inlineStr">
-        <is>
-          <t>ANEXO: la hoja 'Unitarias Basicas' contiene 10 pruebas unitarias básicas adicionales (UNIT-B01 a UNIT-B10) para la entrega del aprendiz.</t>
-        </is>
-      </c>
-    </row>
+    <row r="26" ht="15.75" customHeight="1" s="45"/>
     <row r="27" ht="15.75" customHeight="1" s="45"/>
     <row r="28" ht="15.75" customHeight="1" s="45"/>
     <row r="29" ht="15.75" customHeight="1" s="45"/>
@@ -2333,7 +2200,7 @@
     <row r="999" ht="15.75" customHeight="1" s="45"/>
     <row r="1000" ht="15.75" customHeight="1" s="45"/>
   </sheetData>
-  <mergeCells count="45">
+  <mergeCells count="44">
     <mergeCell ref="F4:G4"/>
     <mergeCell ref="A12:B13"/>
     <mergeCell ref="A1:J2"/>
@@ -2376,7 +2243,6 @@
     <mergeCell ref="A19:B19"/>
     <mergeCell ref="H4:J4"/>
     <mergeCell ref="C4:E4"/>
-    <mergeCell ref="A26:J26"/>
     <mergeCell ref="F24:H24"/>
     <mergeCell ref="H6:J6"/>
   </mergeCells>
@@ -2456,7 +2322,7 @@
       </c>
       <c r="B5" s="48" t="n"/>
       <c r="C5" s="14">
-        <f>COUNTA(A8:A52)</f>
+        <f>COUNTA(A8:A17)</f>
         <v/>
       </c>
       <c r="D5" s="15" t="inlineStr">
@@ -2466,7 +2332,7 @@
       </c>
       <c r="E5" s="48" t="n"/>
       <c r="F5" s="14">
-        <f>COUNTIF(I8:I52,"Exitoso")</f>
+        <f>COUNTIF(I8:I17,"Exitoso")</f>
         <v/>
       </c>
       <c r="G5" s="15" t="inlineStr">
@@ -2476,7 +2342,7 @@
       </c>
       <c r="H5" s="48" t="n"/>
       <c r="I5" s="14">
-        <f>COUNTIF(I8:I52,"Falló")</f>
+        <f>COUNTIF(I8:I17,"Falló")</f>
         <v/>
       </c>
       <c r="J5" s="15" t="inlineStr">
@@ -2484,7 +2350,7 @@
           <t>Tasa de Éxito:</t>
         </is>
       </c>
-      <c r="K5" s="60">
+      <c r="K5" s="65">
         <f>IF(C5&gt;0, F5/C5, 0)</f>
         <v/>
       </c>
@@ -2552,7 +2418,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="120" customHeight="1" s="45">
+    <row r="8" ht="78" customHeight="1" s="45">
       <c r="A8" s="61" t="inlineStr">
         <is>
           <t>UNIT-01</t>
@@ -2560,42 +2426,38 @@
       </c>
       <c r="B8" s="62" t="inlineStr">
         <is>
-          <t>Validadores de registro (api/utils/validators.py): email, teléfono, contraseña y nombre</t>
+          <t>Validación de email: caso válido</t>
         </is>
       </c>
       <c r="C8" s="62" t="inlineStr">
         <is>
-          <t>Módulo importado sin base de datos. Entorno pytest-django con SECRET_KEY de prueba.</t>
+          <t>Función validate_email importada; sin BD ni servidor.</t>
         </is>
       </c>
       <c r="D8" s="62" t="inlineStr">
         <is>
-          <t>email="usuario@plomaap.com" (válido) / "usuario@" (inválido)
-phone="3229874810" (válido) / "123" (inválido)
-password="PlomApp2026*" (válida) / "1234567" (inválida)
-name="Andrés" (válido) / "A" (inválido)</t>
+          <t>email="usuario@plomaap.com"</t>
         </is>
       </c>
       <c r="E8" s="62" t="inlineStr">
         <is>
-          <t>1. Invocar validate_email, validate_phone, validate_password y validate_name con cada dato.
-2. Capturar el valor booleano retornado.
-3. Comparar contra el oráculo.</t>
+          <t>1. Llamar validate_email(email).
+2. Capturar el valor booleano.</t>
         </is>
       </c>
       <c r="F8" s="62" t="inlineStr">
         <is>
-          <t>Datos válidos retornan True; datos inválidos retornan False. Sin excepciones.</t>
+          <t>Retorna True.</t>
         </is>
       </c>
       <c r="G8" s="62" t="inlineStr">
         <is>
-          <t>Aprobado: 23/23 casos parametrizados (email, teléfono, contraseña, nombre y fecha/hora).</t>
+          <t>Aprobado: retornó True.</t>
         </is>
       </c>
       <c r="H8" s="61" t="inlineStr">
         <is>
-          <t>Caja Blanca (Particiones equivalentes + BVA)</t>
+          <t>Caja Blanca (Partición equivalente)</t>
         </is>
       </c>
       <c r="I8" s="61" t="inlineStr">
@@ -2605,362 +2467,586 @@
       </c>
       <c r="J8" s="61" t="inlineStr">
         <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="K8" s="63" t="inlineStr">
+        <is>
+          <t>pytest api\tests\unit\test_unit_10_basicas.py -v: 10 passed; test_01_email_valido</t>
+        </is>
+      </c>
+      <c r="L8" s="62" t="inlineStr">
+        <is>
+          <t>Sin defectos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="78" customHeight="1" s="45">
+      <c r="A9" s="61" t="inlineStr">
+        <is>
+          <t>UNIT-02</t>
+        </is>
+      </c>
+      <c r="B9" s="62" t="inlineStr">
+        <is>
+          <t>Validación de email: caso inválido</t>
+        </is>
+      </c>
+      <c r="C9" s="62" t="inlineStr">
+        <is>
+          <t>Función validate_email importada; sin BD ni servidor.</t>
+        </is>
+      </c>
+      <c r="D9" s="62" t="inlineStr">
+        <is>
+          <t>email="usuario@"</t>
+        </is>
+      </c>
+      <c r="E9" s="62" t="inlineStr">
+        <is>
+          <t>1. Llamar validate_email(email).
+2. Capturar el valor booleano.</t>
+        </is>
+      </c>
+      <c r="F9" s="62" t="inlineStr">
+        <is>
+          <t>Retorna False.</t>
+        </is>
+      </c>
+      <c r="G9" s="62" t="inlineStr">
+        <is>
+          <t>Aprobado: retornó False.</t>
+        </is>
+      </c>
+      <c r="H9" s="61" t="inlineStr">
+        <is>
+          <t>Caja Blanca (Partición equivalente)</t>
+        </is>
+      </c>
+      <c r="I9" s="61" t="inlineStr">
+        <is>
+          <t>Exitoso</t>
+        </is>
+      </c>
+      <c r="J9" s="61" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="K9" s="63" t="inlineStr">
+        <is>
+          <t>pytest api\tests\unit\test_unit_10_basicas.py -v: 10 passed; test_02_email_invalido</t>
+        </is>
+      </c>
+      <c r="L9" s="62" t="inlineStr">
+        <is>
+          <t>Sin defectos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="78" customHeight="1" s="45">
+      <c r="A10" s="61" t="inlineStr">
+        <is>
+          <t>UNIT-03</t>
+        </is>
+      </c>
+      <c r="B10" s="62" t="inlineStr">
+        <is>
+          <t>Validación de teléfono: caso válido</t>
+        </is>
+      </c>
+      <c r="C10" s="62" t="inlineStr">
+        <is>
+          <t>Función validate_phone importada; sin BD ni servidor.</t>
+        </is>
+      </c>
+      <c r="D10" s="62" t="inlineStr">
+        <is>
+          <t>telefono="3229874810"</t>
+        </is>
+      </c>
+      <c r="E10" s="62" t="inlineStr">
+        <is>
+          <t>1. Llamar validate_phone(telefono).
+2. Capturar el valor booleano.</t>
+        </is>
+      </c>
+      <c r="F10" s="62" t="inlineStr">
+        <is>
+          <t>Retorna True.</t>
+        </is>
+      </c>
+      <c r="G10" s="62" t="inlineStr">
+        <is>
+          <t>Aprobado: retornó True.</t>
+        </is>
+      </c>
+      <c r="H10" s="61" t="inlineStr">
+        <is>
+          <t>Caja Blanca (Partición equivalente)</t>
+        </is>
+      </c>
+      <c r="I10" s="61" t="inlineStr">
+        <is>
+          <t>Exitoso</t>
+        </is>
+      </c>
+      <c r="J10" s="61" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="K10" s="63" t="inlineStr">
+        <is>
+          <t>pytest api\tests\unit\test_unit_10_basicas.py -v: 10 passed; test_03_telefono_valido</t>
+        </is>
+      </c>
+      <c r="L10" s="62" t="inlineStr">
+        <is>
+          <t>Sin defectos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="78" customHeight="1" s="45">
+      <c r="A11" s="61" t="inlineStr">
+        <is>
+          <t>UNIT-04</t>
+        </is>
+      </c>
+      <c r="B11" s="62" t="inlineStr">
+        <is>
+          <t>Validación de teléfono: caso inválido</t>
+        </is>
+      </c>
+      <c r="C11" s="62" t="inlineStr">
+        <is>
+          <t>Función validate_phone importada; sin BD ni servidor.</t>
+        </is>
+      </c>
+      <c r="D11" s="62" t="inlineStr">
+        <is>
+          <t>telefono="123"</t>
+        </is>
+      </c>
+      <c r="E11" s="62" t="inlineStr">
+        <is>
+          <t>1. Llamar validate_phone(telefono).
+2. Capturar el valor booleano.</t>
+        </is>
+      </c>
+      <c r="F11" s="62" t="inlineStr">
+        <is>
+          <t>Retorna False.</t>
+        </is>
+      </c>
+      <c r="G11" s="62" t="inlineStr">
+        <is>
+          <t>Aprobado: retornó False.</t>
+        </is>
+      </c>
+      <c r="H11" s="61" t="inlineStr">
+        <is>
+          <t>Caja Blanca (Partición equivalente)</t>
+        </is>
+      </c>
+      <c r="I11" s="61" t="inlineStr">
+        <is>
+          <t>Exitoso</t>
+        </is>
+      </c>
+      <c r="J11" s="61" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="K11" s="63" t="inlineStr">
+        <is>
+          <t>pytest api\tests\unit\test_unit_10_basicas.py -v: 10 passed; test_04_telefono_invalido</t>
+        </is>
+      </c>
+      <c r="L11" s="62" t="inlineStr">
+        <is>
+          <t>Sin defectos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="78" customHeight="1" s="45">
+      <c r="A12" s="61" t="inlineStr">
+        <is>
+          <t>UNIT-05</t>
+        </is>
+      </c>
+      <c r="B12" s="62" t="inlineStr">
+        <is>
+          <t>Validación de contraseña: caso válido</t>
+        </is>
+      </c>
+      <c r="C12" s="62" t="inlineStr">
+        <is>
+          <t>Función validate_password importada; sin BD ni servidor.</t>
+        </is>
+      </c>
+      <c r="D12" s="62" t="inlineStr">
+        <is>
+          <t>password="PlomApp2026*"</t>
+        </is>
+      </c>
+      <c r="E12" s="62" t="inlineStr">
+        <is>
+          <t>1. Llamar validate_password(password).
+2. Capturar el valor booleano.</t>
+        </is>
+      </c>
+      <c r="F12" s="62" t="inlineStr">
+        <is>
+          <t>Retorna True (8 caracteres o más).</t>
+        </is>
+      </c>
+      <c r="G12" s="62" t="inlineStr">
+        <is>
+          <t>Aprobado: retornó True.</t>
+        </is>
+      </c>
+      <c r="H12" s="61" t="inlineStr">
+        <is>
+          <t>Caja Blanca (Valor límite / partición)</t>
+        </is>
+      </c>
+      <c r="I12" s="61" t="inlineStr">
+        <is>
+          <t>Exitoso</t>
+        </is>
+      </c>
+      <c r="J12" s="61" t="inlineStr">
+        <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="K8" s="63" t="inlineStr">
-        <is>
-          <t>pytest -m unit: 35 passed; api/tests/unit/test_unit_01_validators.py</t>
-        </is>
-      </c>
-      <c r="L8" s="62" t="inlineStr">
-        <is>
-          <t>Ejecutado el 26/10/2026 en SQLite en memoria; sin defectos.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="120" customHeight="1" s="45">
-      <c r="A9" s="61" t="inlineStr">
-        <is>
-          <t>UNIT-02</t>
-        </is>
-      </c>
-      <c r="B9" s="62" t="inlineStr">
-        <is>
-          <t>JWT HS256 (api/utils/jwt_utils.py): generación, expiración y firma alterada</t>
-        </is>
-      </c>
-      <c r="C9" s="62" t="inlineStr">
-        <is>
-          <t>settings.JWT_SECRET_KEY y JWT_ALGORITHM=HS256 configurados; freezegun disponible.</t>
-        </is>
-      </c>
-      <c r="D9" s="62" t="inlineStr">
-        <is>
-          <t>user_id=1
-Token válido generado con generate_token(1)
-Token expirado: exp en el pasado
-Token alterado: modificar un carácter de la firma</t>
-        </is>
-      </c>
-      <c r="E9" s="62" t="inlineStr">
-        <is>
-          <t>1. Generar token con generate_token(1).
-2. Decodificar con decode_token.
-3. Repetir con token expirado y con firma alterada.</t>
-        </is>
-      </c>
-      <c r="F9" s="62" t="inlineStr">
-        <is>
-          <t>Token válido: payload con sub="1" (string), iat y exp.
-Token expirado o alterado: decode_token retorna None, sin excepción no controlada.</t>
-        </is>
-      </c>
-      <c r="G9" s="62" t="inlineStr">
-        <is>
-          <t>Aprobado: 4/4 casos (token válido con sub string, expiración, firma alterada y token inválido).</t>
-        </is>
-      </c>
-      <c r="H9" s="61" t="inlineStr">
-        <is>
-          <t>Caja Blanca (Seguridad / caminos de error)</t>
-        </is>
-      </c>
-      <c r="I9" s="61" t="inlineStr">
+      <c r="K12" s="63" t="inlineStr">
+        <is>
+          <t>pytest api\tests\unit\test_unit_10_basicas.py -v: 10 passed; test_05_password_valido</t>
+        </is>
+      </c>
+      <c r="L12" s="62" t="inlineStr">
+        <is>
+          <t>Sin defectos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="78" customHeight="1" s="45">
+      <c r="A13" s="61" t="inlineStr">
+        <is>
+          <t>UNIT-06</t>
+        </is>
+      </c>
+      <c r="B13" s="62" t="inlineStr">
+        <is>
+          <t>Validación de contraseña: caso corto</t>
+        </is>
+      </c>
+      <c r="C13" s="62" t="inlineStr">
+        <is>
+          <t>Función validate_password importada; sin BD ni servidor.</t>
+        </is>
+      </c>
+      <c r="D13" s="62" t="inlineStr">
+        <is>
+          <t>password="1234567"</t>
+        </is>
+      </c>
+      <c r="E13" s="62" t="inlineStr">
+        <is>
+          <t>1. Llamar validate_password(password).
+2. Capturar el valor booleano.</t>
+        </is>
+      </c>
+      <c r="F13" s="62" t="inlineStr">
+        <is>
+          <t>Retorna False (7 caracteres).</t>
+        </is>
+      </c>
+      <c r="G13" s="62" t="inlineStr">
+        <is>
+          <t>Aprobado: retornó False.</t>
+        </is>
+      </c>
+      <c r="H13" s="61" t="inlineStr">
+        <is>
+          <t>Caja Blanca (Valor límite / partición)</t>
+        </is>
+      </c>
+      <c r="I13" s="61" t="inlineStr">
         <is>
           <t>Exitoso</t>
         </is>
       </c>
-      <c r="J9" s="61" t="inlineStr">
+      <c r="J13" s="61" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="K9" s="63" t="inlineStr">
-        <is>
-          <t>pytest -m unit: 35 passed; api/tests/unit/test_unit_02_jwt.py</t>
-        </is>
-      </c>
-      <c r="L9" s="62" t="inlineStr">
-        <is>
-          <t>Ejecutado el 26/10/2026; se verificó compatibilidad HS256 con el contrato Flask.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="120" customHeight="1" s="45">
-      <c r="A10" s="61" t="inlineStr">
-        <is>
-          <t>UNIT-03</t>
-        </is>
-      </c>
-      <c r="B10" s="62" t="inlineStr">
-        <is>
-          <t>Disponibilidad de citas (api/services/appointment_service.py): get_smart_time_slots y validate_appointment_transition</t>
-        </is>
-      </c>
-      <c r="C10" s="62" t="inlineStr">
-        <is>
-          <t>BD de prueba con servicio de 60 min y técnico activo con schedule {"mon": [[8,18]]}; freezegun para fijar la fecha.</t>
-        </is>
-      </c>
-      <c r="D10" s="62" t="inlineStr">
-        <is>
-          <t>date="2026-11-02" (lunes), service_id=1, technician_id=1
-Sin citas: todos los slots 08:00-17:00 disponibles.
-Con cita 09:00: slot 09:00 no disponible.
-Hoy a las 17:45: slots antes de 18:15 no disponibles.
-Transiciones: scheduled-&gt;in_progress (válida), completed-&gt;scheduled (inválida).</t>
-        </is>
-      </c>
-      <c r="E10" s="62" t="inlineStr">
-        <is>
-          <t>1. Ejecutar get_smart_time_slots(1, "2026-11-02", 1).
-2. Crear cita en 09:00 y repetir.
-3. Congelar hora en 17:45 y consultar el mismo día.
-4. Evaluar validate_appointment_transition.</t>
-        </is>
-      </c>
-      <c r="F10" s="62" t="inlineStr">
-        <is>
-          <t>Slots de 08:00 a 17:00 con available=True; 09:00 con available=False tras la cita; ningún slot pasado hoy; transiciones válidas=True e inválidas=False.</t>
-        </is>
-      </c>
-      <c r="G10" s="62" t="inlineStr">
-        <is>
-          <t>Aprobado: 3/3 pruebas (10 slots, conflicto 09:00, hoy sin slots pasados y transiciones de estado).</t>
-        </is>
-      </c>
-      <c r="H10" s="61" t="inlineStr">
-        <is>
-          <t>Caja Blanca (BVA / reglas de negocio)</t>
-        </is>
-      </c>
-      <c r="I10" s="61" t="inlineStr">
+      <c r="K13" s="63" t="inlineStr">
+        <is>
+          <t>pytest api\tests\unit\test_unit_10_basicas.py -v: 10 passed; test_06_password_corto</t>
+        </is>
+      </c>
+      <c r="L13" s="62" t="inlineStr">
+        <is>
+          <t>Sin defectos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="78" customHeight="1" s="45">
+      <c r="A14" s="61" t="inlineStr">
+        <is>
+          <t>UNIT-07</t>
+        </is>
+      </c>
+      <c r="B14" s="62" t="inlineStr">
+        <is>
+          <t>Validación de nombre: caso válido</t>
+        </is>
+      </c>
+      <c r="C14" s="62" t="inlineStr">
+        <is>
+          <t>Función validate_name importada; sin BD ni servidor.</t>
+        </is>
+      </c>
+      <c r="D14" s="62" t="inlineStr">
+        <is>
+          <t>nombre="Andrés"</t>
+        </is>
+      </c>
+      <c r="E14" s="62" t="inlineStr">
+        <is>
+          <t>1. Llamar validate_name(nombre).
+2. Capturar el valor booleano.</t>
+        </is>
+      </c>
+      <c r="F14" s="62" t="inlineStr">
+        <is>
+          <t>Retorna True (2 caracteres o más).</t>
+        </is>
+      </c>
+      <c r="G14" s="62" t="inlineStr">
+        <is>
+          <t>Aprobado: retornó True.</t>
+        </is>
+      </c>
+      <c r="H14" s="61" t="inlineStr">
+        <is>
+          <t>Caja Blanca (Partición equivalente)</t>
+        </is>
+      </c>
+      <c r="I14" s="61" t="inlineStr">
         <is>
           <t>Exitoso</t>
         </is>
       </c>
-      <c r="J10" s="61" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="K10" s="63" t="inlineStr">
-        <is>
-          <t>pytest -m unit: 35 passed; api/tests/unit/test_unit_03_appointment_slots.py</t>
-        </is>
-      </c>
-      <c r="L10" s="62" t="inlineStr">
-        <is>
-          <t>Ejecutado el 26/10/2026 con freezegun; sin defectos.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="120" customHeight="1" s="45">
-      <c r="A11" s="61" t="inlineStr">
-        <is>
-          <t>UNIT-04</t>
-        </is>
-      </c>
-      <c r="B11" s="62" t="inlineStr">
-        <is>
-          <t>Matemática de embeddings (api/services/embedding_service.py): _parse_vector y _cosine_similarity</t>
-        </is>
-      </c>
-      <c r="C11" s="62" t="inlineStr">
-        <is>
-          <t>Funciones puras importadas; sin BD ni proveedor externo.</t>
-        </is>
-      </c>
-      <c r="D11" s="62" t="inlineStr">
-        <is>
-          <t>_parse_vector("[1.0, 2.0, 3.0]") -&gt; [1.0, 2.0, 3.0]
-_parse_vector("abc") -&gt; None
-_cosine_similarity([1,0,0], [1,0,0]) -&gt; 1.0
-_cosine_similarity([1,0,0], [0,1,0]) -&gt; 0.0
-_cosine_similarity([], []) -&gt; 0.0
-_cosine_similarity([1,0], [1,0,0]) -&gt; 0.0</t>
-        </is>
-      </c>
-      <c r="E11" s="62" t="inlineStr">
-        <is>
-          <t>1. Invocar _parse_vector con JSON válido e inválido.
-2. Invocar _cosine_similarity con vectores iguales, ortogonales, vacíos y de distinta dimensión.</t>
-        </is>
-      </c>
-      <c r="F11" s="62" t="inlineStr">
-        <is>
-          <t>Parseo correcto de listas; None para texto inválido; similitud 1.0, 0.0 y 0.0 en los casos límite; sin ZeroDivisionError.</t>
-        </is>
-      </c>
-      <c r="G11" s="62" t="inlineStr">
-        <is>
-          <t>Aprobado: 5/5 casos (parseo válido/inválido, coseno 1.0, 0.0 y casos límite).</t>
-        </is>
-      </c>
-      <c r="H11" s="61" t="inlineStr">
-        <is>
-          <t>Caja Blanca (Frontera / casos límite)</t>
-        </is>
-      </c>
-      <c r="I11" s="61" t="inlineStr">
+      <c r="J14" s="61" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="K14" s="63" t="inlineStr">
+        <is>
+          <t>pytest api\tests\unit\test_unit_10_basicas.py -v: 10 passed; test_07_nombre_valido</t>
+        </is>
+      </c>
+      <c r="L14" s="62" t="inlineStr">
+        <is>
+          <t>Sin defectos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="78" customHeight="1" s="45">
+      <c r="A15" s="61" t="inlineStr">
+        <is>
+          <t>UNIT-08</t>
+        </is>
+      </c>
+      <c r="B15" s="62" t="inlineStr">
+        <is>
+          <t>Validación de nombre: caso corto</t>
+        </is>
+      </c>
+      <c r="C15" s="62" t="inlineStr">
+        <is>
+          <t>Función validate_name importada; sin BD ni servidor.</t>
+        </is>
+      </c>
+      <c r="D15" s="62" t="inlineStr">
+        <is>
+          <t>nombre="A"</t>
+        </is>
+      </c>
+      <c r="E15" s="62" t="inlineStr">
+        <is>
+          <t>1. Llamar validate_name(nombre).
+2. Capturar el valor booleano.</t>
+        </is>
+      </c>
+      <c r="F15" s="62" t="inlineStr">
+        <is>
+          <t>Retorna False (1 carácter).</t>
+        </is>
+      </c>
+      <c r="G15" s="62" t="inlineStr">
+        <is>
+          <t>Aprobado: retornó False.</t>
+        </is>
+      </c>
+      <c r="H15" s="61" t="inlineStr">
+        <is>
+          <t>Caja Blanca (Valor límite / partición)</t>
+        </is>
+      </c>
+      <c r="I15" s="61" t="inlineStr">
         <is>
           <t>Exitoso</t>
         </is>
       </c>
-      <c r="J11" s="61" t="inlineStr">
+      <c r="J15" s="61" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="K11" s="63" t="inlineStr">
-        <is>
-          <t>pytest -m unit: 35 passed; api/tests/unit/test_unit_04_embedding_math.py</t>
-        </is>
-      </c>
-      <c r="L11" s="62" t="inlineStr">
-        <is>
-          <t>Ejecutado el 26/10/2026; no requiere pgvector ni red.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="120" customHeight="1" s="45">
-      <c r="A12" s="61" t="inlineStr">
-        <is>
-          <t>UNIT-05</t>
-        </is>
-      </c>
-      <c r="B12" s="62" t="inlineStr">
-        <is>
-          <t>Validaciones del frontend (src/utils/validation.js): email, teléfono y nombre</t>
-        </is>
-      </c>
-      <c r="C12" s="62" t="inlineStr">
-        <is>
-          <t>Vitest + jsdom configurados; módulo validation.js importado.</t>
-        </is>
-      </c>
-      <c r="D12" s="62" t="inlineStr">
-        <is>
-          <t>validateEmail("usuario@plomaap.com") -&gt; ""
-validateEmail("usuario@") -&gt; mensaje de error
-validatePhone("3229874810") -&gt; ""
-validatePhone("12345") -&gt; mensaje de error
-validateName("Andrés Pérez") -&gt; ""
-validateName("Andrés") -&gt; mensaje de error</t>
-        </is>
-      </c>
-      <c r="E12" s="62" t="inlineStr">
-        <is>
-          <t>1. Ejecutar cada validador con datos válidos e inválidos.
-2. Comparar el string retornado contra MESSAGES.</t>
-        </is>
-      </c>
-      <c r="F12" s="62" t="inlineStr">
-        <is>
-          <t>Datos válidos retornan cadena vacía; inválidos retornan el mensaje correspondiente de MESSAGES; sin excepciones.</t>
-        </is>
-      </c>
-      <c r="G12" s="62" t="inlineStr">
-        <is>
-          <t>Aprobado: 6/6 pruebas Vitest (email, nombre, teléfono, contraseña, registro y login).</t>
-        </is>
-      </c>
-      <c r="H12" s="61" t="inlineStr">
-        <is>
-          <t>Caja Negra (Particiones equivalentes / UI)</t>
-        </is>
-      </c>
-      <c r="I12" s="61" t="inlineStr">
+      <c r="K15" s="63" t="inlineStr">
+        <is>
+          <t>pytest api\tests\unit\test_unit_10_basicas.py -v: 10 passed; test_08_nombre_corto</t>
+        </is>
+      </c>
+      <c r="L15" s="62" t="inlineStr">
+        <is>
+          <t>Sin defectos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="78" customHeight="1" s="45">
+      <c r="A16" s="61" t="inlineStr">
+        <is>
+          <t>UNIT-09</t>
+        </is>
+      </c>
+      <c r="B16" s="62" t="inlineStr">
+        <is>
+          <t>Validación de fecha y hora: caso válido</t>
+        </is>
+      </c>
+      <c r="C16" s="62" t="inlineStr">
+        <is>
+          <t>Función validate_date_time importada; sin BD ni servidor.</t>
+        </is>
+      </c>
+      <c r="D16" s="62" t="inlineStr">
+        <is>
+          <t>fecha="2026-11-02" / hora="09:00"</t>
+        </is>
+      </c>
+      <c r="E16" s="62" t="inlineStr">
+        <is>
+          <t>1. Llamar validate_date_time(fecha, hora).
+2. Capturar el valor booleano.</t>
+        </is>
+      </c>
+      <c r="F16" s="62" t="inlineStr">
+        <is>
+          <t>Retorna True.</t>
+        </is>
+      </c>
+      <c r="G16" s="62" t="inlineStr">
+        <is>
+          <t>Aprobado: retornó True.</t>
+        </is>
+      </c>
+      <c r="H16" s="61" t="inlineStr">
+        <is>
+          <t>Caja Blanca (Formato / partición)</t>
+        </is>
+      </c>
+      <c r="I16" s="61" t="inlineStr">
         <is>
           <t>Exitoso</t>
         </is>
       </c>
-      <c r="J12" s="61" t="inlineStr">
+      <c r="J16" s="61" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="K12" s="63" t="inlineStr">
-        <is>
-          <t>npm run test:unit: 6 passed; tests/unit/unit_05_validation.test.js</t>
-        </is>
-      </c>
-      <c r="L12" s="62" t="inlineStr">
-        <is>
-          <t>Ejecutado el 26/10/2026 con Vitest 5.0.5 + jsdom 29.1.1.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="25.5" customHeight="1" s="45">
-      <c r="A13" s="22" t="n"/>
-      <c r="B13" s="23" t="n"/>
-      <c r="C13" s="23" t="n"/>
-      <c r="D13" s="23" t="n"/>
-      <c r="E13" s="23" t="n"/>
-      <c r="F13" s="23" t="n"/>
-      <c r="G13" s="23" t="n"/>
-      <c r="H13" s="22" t="n"/>
-      <c r="I13" s="22" t="n"/>
-      <c r="J13" s="22" t="n"/>
-      <c r="K13" s="23" t="n"/>
-      <c r="L13" s="23" t="n"/>
-    </row>
-    <row r="14" ht="25.5" customHeight="1" s="45">
-      <c r="A14" s="27" t="n"/>
-      <c r="B14" s="28" t="n"/>
-      <c r="C14" s="28" t="n"/>
-      <c r="D14" s="28" t="n"/>
-      <c r="E14" s="28" t="n"/>
-      <c r="F14" s="28" t="n"/>
-      <c r="G14" s="28" t="n"/>
-      <c r="H14" s="27" t="n"/>
-      <c r="I14" s="27" t="n"/>
-      <c r="J14" s="27" t="n"/>
-      <c r="K14" s="28" t="n"/>
-      <c r="L14" s="28" t="n"/>
-    </row>
-    <row r="15" ht="25.5" customHeight="1" s="45">
-      <c r="A15" s="22" t="n"/>
-      <c r="B15" s="23" t="n"/>
-      <c r="C15" s="23" t="n"/>
-      <c r="D15" s="23" t="n"/>
-      <c r="E15" s="23" t="n"/>
-      <c r="F15" s="23" t="n"/>
-      <c r="G15" s="23" t="n"/>
-      <c r="H15" s="22" t="n"/>
-      <c r="I15" s="22" t="n"/>
-      <c r="J15" s="22" t="n"/>
-      <c r="K15" s="23" t="n"/>
-      <c r="L15" s="23" t="n"/>
-    </row>
-    <row r="16" ht="25.5" customHeight="1" s="45">
-      <c r="A16" s="27" t="n"/>
-      <c r="B16" s="28" t="n"/>
-      <c r="C16" s="28" t="n"/>
-      <c r="D16" s="28" t="n"/>
-      <c r="E16" s="28" t="n"/>
-      <c r="F16" s="28" t="n"/>
-      <c r="G16" s="28" t="n"/>
-      <c r="H16" s="27" t="n"/>
-      <c r="I16" s="27" t="n"/>
-      <c r="J16" s="27" t="n"/>
-      <c r="K16" s="28" t="n"/>
-      <c r="L16" s="28" t="n"/>
-    </row>
-    <row r="17" ht="25.5" customHeight="1" s="45">
-      <c r="A17" s="22" t="n"/>
-      <c r="B17" s="23" t="n"/>
-      <c r="C17" s="23" t="n"/>
-      <c r="D17" s="23" t="n"/>
-      <c r="E17" s="23" t="n"/>
-      <c r="F17" s="23" t="n"/>
-      <c r="G17" s="23" t="n"/>
-      <c r="H17" s="22" t="n"/>
-      <c r="I17" s="22" t="n"/>
-      <c r="J17" s="22" t="n"/>
-      <c r="K17" s="23" t="n"/>
-      <c r="L17" s="23" t="n"/>
+      <c r="K16" s="63" t="inlineStr">
+        <is>
+          <t>pytest api\tests\unit\test_unit_10_basicas.py -v: 10 passed; test_09_fecha_y_hora_validas</t>
+        </is>
+      </c>
+      <c r="L16" s="62" t="inlineStr">
+        <is>
+          <t>Sin defectos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="78" customHeight="1" s="45">
+      <c r="A17" s="61" t="inlineStr">
+        <is>
+          <t>UNIT-10</t>
+        </is>
+      </c>
+      <c r="B17" s="62" t="inlineStr">
+        <is>
+          <t>Validación de fecha y hora: caso inválido</t>
+        </is>
+      </c>
+      <c r="C17" s="62" t="inlineStr">
+        <is>
+          <t>Función validate_date_time importada; sin BD ni servidor.</t>
+        </is>
+      </c>
+      <c r="D17" s="62" t="inlineStr">
+        <is>
+          <t>fecha="2026-13-01" / hora="09:00"</t>
+        </is>
+      </c>
+      <c r="E17" s="62" t="inlineStr">
+        <is>
+          <t>1. Llamar validate_date_time(fecha, hora).
+2. Capturar el valor booleano.</t>
+        </is>
+      </c>
+      <c r="F17" s="62" t="inlineStr">
+        <is>
+          <t>Retorna False (mes 13 inexistente).</t>
+        </is>
+      </c>
+      <c r="G17" s="62" t="inlineStr">
+        <is>
+          <t>Aprobado: retornó False.</t>
+        </is>
+      </c>
+      <c r="H17" s="61" t="inlineStr">
+        <is>
+          <t>Caja Blanca (Valor inválido / formato)</t>
+        </is>
+      </c>
+      <c r="I17" s="61" t="inlineStr">
+        <is>
+          <t>Exitoso</t>
+        </is>
+      </c>
+      <c r="J17" s="61" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="K17" s="63" t="inlineStr">
+        <is>
+          <t>pytest api\tests\unit\test_unit_10_basicas.py -v: 10 passed; test_10_fecha_y_hora_invalida</t>
+        </is>
+      </c>
+      <c r="L17" s="62" t="inlineStr">
+        <is>
+          <t>Sin defectos.</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="25.5" customHeight="1" s="45">
       <c r="A18" s="27" t="n"/>
@@ -9360,793 +9446,4 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:L19"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" style="45" min="1" max="1"/>
-    <col width="34" customWidth="1" style="45" min="2" max="2"/>
-    <col width="32" customWidth="1" style="45" min="3" max="3"/>
-    <col width="36" customWidth="1" style="45" min="4" max="4"/>
-    <col width="40" customWidth="1" style="45" min="5" max="5"/>
-    <col width="40" customWidth="1" style="45" min="6" max="6"/>
-    <col width="36" customWidth="1" style="45" min="7" max="7"/>
-    <col width="24" customWidth="1" style="45" min="8" max="8"/>
-    <col width="12" customWidth="1" style="45" min="9" max="9"/>
-    <col width="11" customWidth="1" style="45" min="10" max="10"/>
-    <col width="42" customWidth="1" style="45" min="11" max="11"/>
-    <col width="34" customWidth="1" style="45" min="12" max="12"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="32" customHeight="1" s="45">
-      <c r="A1" s="66" t="inlineStr">
-        <is>
-          <t>SENA - SIGA | ANEXO: 10 PRUEBAS UNITARIAS BÁSICAS (ENTREGA DEL APRENDIZ)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="67" t="inlineStr">
-        <is>
-          <t>Nivel de Prueba:</t>
-        </is>
-      </c>
-      <c r="C3" s="68" t="inlineStr">
-        <is>
-          <t>Nivel 1: Pruebas Unitarias (Unit Testing) - validadores puros</t>
-        </is>
-      </c>
-      <c r="G3" s="67" t="inlineStr">
-        <is>
-          <t>Enfoque:</t>
-        </is>
-      </c>
-      <c r="I3" s="68" t="inlineStr">
-        <is>
-          <t>Funciones de api/utils/validators.py; sin base de datos, servidor ni internet.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="67" t="inlineStr">
-        <is>
-          <t>Total Ejecutadas:</t>
-        </is>
-      </c>
-      <c r="B5" s="69" t="n">
-        <v>10</v>
-      </c>
-      <c r="C5" s="67" t="inlineStr">
-        <is>
-          <t>Exitosas (Aprobadas):</t>
-        </is>
-      </c>
-      <c r="D5" s="69" t="n">
-        <v>10</v>
-      </c>
-      <c r="E5" s="67" t="inlineStr">
-        <is>
-          <t>Fallidas (Defectos):</t>
-        </is>
-      </c>
-      <c r="F5" s="69" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" s="67" t="inlineStr">
-        <is>
-          <t>Tasa de Éxito:</t>
-        </is>
-      </c>
-      <c r="H5" s="70" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" ht="44" customHeight="1" s="45">
-      <c r="A7" s="71" t="inlineStr">
-        <is>
-          <t>ID Caso</t>
-        </is>
-      </c>
-      <c r="B7" s="71" t="inlineStr">
-        <is>
-          <t>Componente / Escenario Probado</t>
-        </is>
-      </c>
-      <c r="C7" s="71" t="inlineStr">
-        <is>
-          <t>Precondiciones / Configuración</t>
-        </is>
-      </c>
-      <c r="D7" s="71" t="inlineStr">
-        <is>
-          <t>Datos de Entrada (Arrange)</t>
-        </is>
-      </c>
-      <c r="E7" s="71" t="inlineStr">
-        <is>
-          <t>Pasos de Ejecución (Act)</t>
-        </is>
-      </c>
-      <c r="F7" s="71" t="inlineStr">
-        <is>
-          <t>Resultado Esperado (Assert / Oráculo)</t>
-        </is>
-      </c>
-      <c r="G7" s="71" t="inlineStr">
-        <is>
-          <t>Resultado Obtenido en Ejecución</t>
-        </is>
-      </c>
-      <c r="H7" s="71" t="inlineStr">
-        <is>
-          <t>Tipo / Técnica</t>
-        </is>
-      </c>
-      <c r="I7" s="71" t="inlineStr">
-        <is>
-          <t>Estado</t>
-        </is>
-      </c>
-      <c r="J7" s="71" t="inlineStr">
-        <is>
-          <t>Severidad / Prioridad</t>
-        </is>
-      </c>
-      <c r="K7" s="71" t="inlineStr">
-        <is>
-          <t>Evidencia (URL / Test Pass / Log)</t>
-        </is>
-      </c>
-      <c r="L7" s="71" t="inlineStr">
-        <is>
-          <t>Observaciones / Defecto Asociado</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="58" customHeight="1" s="45">
-      <c r="A8" s="72" t="inlineStr">
-        <is>
-          <t>UNIT-B01</t>
-        </is>
-      </c>
-      <c r="B8" s="73" t="inlineStr">
-        <is>
-          <t>Validación de email: caso válido</t>
-        </is>
-      </c>
-      <c r="C8" s="73" t="inlineStr">
-        <is>
-          <t>Función validate_email importada; sin BD ni servidor.</t>
-        </is>
-      </c>
-      <c r="D8" s="73" t="inlineStr">
-        <is>
-          <t>email="usuario@plomaap.com"</t>
-        </is>
-      </c>
-      <c r="E8" s="73" t="inlineStr">
-        <is>
-          <t>1. Llamar validate_email(email). / 2. Capturar el valor booleano.</t>
-        </is>
-      </c>
-      <c r="F8" s="73" t="inlineStr">
-        <is>
-          <t>Retorna True.</t>
-        </is>
-      </c>
-      <c r="G8" s="73" t="inlineStr">
-        <is>
-          <t>Aprobado: retornó True.</t>
-        </is>
-      </c>
-      <c r="H8" s="73" t="inlineStr">
-        <is>
-          <t>Caja Blanca (Partición equivalente)</t>
-        </is>
-      </c>
-      <c r="I8" s="74" t="inlineStr">
-        <is>
-          <t>Exitoso</t>
-        </is>
-      </c>
-      <c r="J8" s="72" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="K8" s="73" t="inlineStr">
-        <is>
-          <t>pytest api\tests\unit\test_unit_10_basicas.py -v: 10 passed; test_01_email_valido</t>
-        </is>
-      </c>
-      <c r="L8" s="73" t="inlineStr">
-        <is>
-          <t>Sin defectos.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="58" customHeight="1" s="45">
-      <c r="A9" s="75" t="inlineStr">
-        <is>
-          <t>UNIT-B02</t>
-        </is>
-      </c>
-      <c r="B9" s="76" t="inlineStr">
-        <is>
-          <t>Validación de email: caso inválido</t>
-        </is>
-      </c>
-      <c r="C9" s="76" t="inlineStr">
-        <is>
-          <t>Función validate_email importada; sin BD ni servidor.</t>
-        </is>
-      </c>
-      <c r="D9" s="76" t="inlineStr">
-        <is>
-          <t>email="usuario@"</t>
-        </is>
-      </c>
-      <c r="E9" s="76" t="inlineStr">
-        <is>
-          <t>1. Llamar validate_email(email). / 2. Capturar el valor booleano.</t>
-        </is>
-      </c>
-      <c r="F9" s="76" t="inlineStr">
-        <is>
-          <t>Retorna False.</t>
-        </is>
-      </c>
-      <c r="G9" s="76" t="inlineStr">
-        <is>
-          <t>Aprobado: retornó False.</t>
-        </is>
-      </c>
-      <c r="H9" s="76" t="inlineStr">
-        <is>
-          <t>Caja Blanca (Partición equivalente)</t>
-        </is>
-      </c>
-      <c r="I9" s="74" t="inlineStr">
-        <is>
-          <t>Exitoso</t>
-        </is>
-      </c>
-      <c r="J9" s="75" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="K9" s="76" t="inlineStr">
-        <is>
-          <t>pytest api\tests\unit\test_unit_10_basicas.py -v: 10 passed; test_02_email_invalido</t>
-        </is>
-      </c>
-      <c r="L9" s="76" t="inlineStr">
-        <is>
-          <t>Sin defectos.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="58" customHeight="1" s="45">
-      <c r="A10" s="72" t="inlineStr">
-        <is>
-          <t>UNIT-B03</t>
-        </is>
-      </c>
-      <c r="B10" s="73" t="inlineStr">
-        <is>
-          <t>Validación de teléfono: caso válido</t>
-        </is>
-      </c>
-      <c r="C10" s="73" t="inlineStr">
-        <is>
-          <t>Función validate_phone importada; sin BD ni servidor.</t>
-        </is>
-      </c>
-      <c r="D10" s="73" t="inlineStr">
-        <is>
-          <t>telefono="3229874810"</t>
-        </is>
-      </c>
-      <c r="E10" s="73" t="inlineStr">
-        <is>
-          <t>1. Llamar validate_phone(telefono). / 2. Capturar el valor booleano.</t>
-        </is>
-      </c>
-      <c r="F10" s="73" t="inlineStr">
-        <is>
-          <t>Retorna True.</t>
-        </is>
-      </c>
-      <c r="G10" s="73" t="inlineStr">
-        <is>
-          <t>Aprobado: retornó True.</t>
-        </is>
-      </c>
-      <c r="H10" s="73" t="inlineStr">
-        <is>
-          <t>Caja Blanca (Partición equivalente)</t>
-        </is>
-      </c>
-      <c r="I10" s="74" t="inlineStr">
-        <is>
-          <t>Exitoso</t>
-        </is>
-      </c>
-      <c r="J10" s="72" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="K10" s="73" t="inlineStr">
-        <is>
-          <t>pytest api\tests\unit\test_unit_10_basicas.py -v: 10 passed; test_03_telefono_valido</t>
-        </is>
-      </c>
-      <c r="L10" s="73" t="inlineStr">
-        <is>
-          <t>Sin defectos.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="58" customHeight="1" s="45">
-      <c r="A11" s="75" t="inlineStr">
-        <is>
-          <t>UNIT-B04</t>
-        </is>
-      </c>
-      <c r="B11" s="76" t="inlineStr">
-        <is>
-          <t>Validación de teléfono: caso inválido</t>
-        </is>
-      </c>
-      <c r="C11" s="76" t="inlineStr">
-        <is>
-          <t>Función validate_phone importada; sin BD ni servidor.</t>
-        </is>
-      </c>
-      <c r="D11" s="76" t="inlineStr">
-        <is>
-          <t>telefono="123"</t>
-        </is>
-      </c>
-      <c r="E11" s="76" t="inlineStr">
-        <is>
-          <t>1. Llamar validate_phone(telefono). / 2. Capturar el valor booleano.</t>
-        </is>
-      </c>
-      <c r="F11" s="76" t="inlineStr">
-        <is>
-          <t>Retorna False.</t>
-        </is>
-      </c>
-      <c r="G11" s="76" t="inlineStr">
-        <is>
-          <t>Aprobado: retornó False.</t>
-        </is>
-      </c>
-      <c r="H11" s="76" t="inlineStr">
-        <is>
-          <t>Caja Blanca (Partición equivalente)</t>
-        </is>
-      </c>
-      <c r="I11" s="74" t="inlineStr">
-        <is>
-          <t>Exitoso</t>
-        </is>
-      </c>
-      <c r="J11" s="75" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="K11" s="76" t="inlineStr">
-        <is>
-          <t>pytest api\tests\unit\test_unit_10_basicas.py -v: 10 passed; test_04_telefono_invalido</t>
-        </is>
-      </c>
-      <c r="L11" s="76" t="inlineStr">
-        <is>
-          <t>Sin defectos.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="58" customHeight="1" s="45">
-      <c r="A12" s="72" t="inlineStr">
-        <is>
-          <t>UNIT-B05</t>
-        </is>
-      </c>
-      <c r="B12" s="73" t="inlineStr">
-        <is>
-          <t>Validación de contraseña: caso válido</t>
-        </is>
-      </c>
-      <c r="C12" s="73" t="inlineStr">
-        <is>
-          <t>Función validate_password importada; sin BD ni servidor.</t>
-        </is>
-      </c>
-      <c r="D12" s="73" t="inlineStr">
-        <is>
-          <t>password="PlomApp2026*"</t>
-        </is>
-      </c>
-      <c r="E12" s="73" t="inlineStr">
-        <is>
-          <t>1. Llamar validate_password(password). / 2. Capturar el valor booleano.</t>
-        </is>
-      </c>
-      <c r="F12" s="73" t="inlineStr">
-        <is>
-          <t>Retorna True (8 caracteres o más).</t>
-        </is>
-      </c>
-      <c r="G12" s="73" t="inlineStr">
-        <is>
-          <t>Aprobado: retornó True.</t>
-        </is>
-      </c>
-      <c r="H12" s="73" t="inlineStr">
-        <is>
-          <t>Caja Blanca (Valor límite / partición)</t>
-        </is>
-      </c>
-      <c r="I12" s="74" t="inlineStr">
-        <is>
-          <t>Exitoso</t>
-        </is>
-      </c>
-      <c r="J12" s="72" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="K12" s="73" t="inlineStr">
-        <is>
-          <t>pytest api\tests\unit\test_unit_10_basicas.py -v: 10 passed; test_05_password_valido</t>
-        </is>
-      </c>
-      <c r="L12" s="73" t="inlineStr">
-        <is>
-          <t>Sin defectos.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="58" customHeight="1" s="45">
-      <c r="A13" s="75" t="inlineStr">
-        <is>
-          <t>UNIT-B06</t>
-        </is>
-      </c>
-      <c r="B13" s="76" t="inlineStr">
-        <is>
-          <t>Validación de contraseña: caso corto</t>
-        </is>
-      </c>
-      <c r="C13" s="76" t="inlineStr">
-        <is>
-          <t>Función validate_password importada; sin BD ni servidor.</t>
-        </is>
-      </c>
-      <c r="D13" s="76" t="inlineStr">
-        <is>
-          <t>password="1234567"</t>
-        </is>
-      </c>
-      <c r="E13" s="76" t="inlineStr">
-        <is>
-          <t>1. Llamar validate_password(password). / 2. Capturar el valor booleano.</t>
-        </is>
-      </c>
-      <c r="F13" s="76" t="inlineStr">
-        <is>
-          <t>Retorna False (7 caracteres).</t>
-        </is>
-      </c>
-      <c r="G13" s="76" t="inlineStr">
-        <is>
-          <t>Aprobado: retornó False.</t>
-        </is>
-      </c>
-      <c r="H13" s="76" t="inlineStr">
-        <is>
-          <t>Caja Blanca (Valor límite / partición)</t>
-        </is>
-      </c>
-      <c r="I13" s="74" t="inlineStr">
-        <is>
-          <t>Exitoso</t>
-        </is>
-      </c>
-      <c r="J13" s="75" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="K13" s="76" t="inlineStr">
-        <is>
-          <t>pytest api\tests\unit\test_unit_10_basicas.py -v: 10 passed; test_06_password_corto</t>
-        </is>
-      </c>
-      <c r="L13" s="76" t="inlineStr">
-        <is>
-          <t>Sin defectos.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="58" customHeight="1" s="45">
-      <c r="A14" s="72" t="inlineStr">
-        <is>
-          <t>UNIT-B07</t>
-        </is>
-      </c>
-      <c r="B14" s="73" t="inlineStr">
-        <is>
-          <t>Validación de nombre: caso válido</t>
-        </is>
-      </c>
-      <c r="C14" s="73" t="inlineStr">
-        <is>
-          <t>Función validate_name importada; sin BD ni servidor.</t>
-        </is>
-      </c>
-      <c r="D14" s="73" t="inlineStr">
-        <is>
-          <t>nombre="Andrés"</t>
-        </is>
-      </c>
-      <c r="E14" s="73" t="inlineStr">
-        <is>
-          <t>1. Llamar validate_name(nombre). / 2. Capturar el valor booleano.</t>
-        </is>
-      </c>
-      <c r="F14" s="73" t="inlineStr">
-        <is>
-          <t>Retorna True (2 caracteres o más).</t>
-        </is>
-      </c>
-      <c r="G14" s="73" t="inlineStr">
-        <is>
-          <t>Aprobado: retornó True.</t>
-        </is>
-      </c>
-      <c r="H14" s="73" t="inlineStr">
-        <is>
-          <t>Caja Blanca (Partición equivalente)</t>
-        </is>
-      </c>
-      <c r="I14" s="74" t="inlineStr">
-        <is>
-          <t>Exitoso</t>
-        </is>
-      </c>
-      <c r="J14" s="72" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="K14" s="73" t="inlineStr">
-        <is>
-          <t>pytest api\tests\unit\test_unit_10_basicas.py -v: 10 passed; test_07_nombre_valido</t>
-        </is>
-      </c>
-      <c r="L14" s="73" t="inlineStr">
-        <is>
-          <t>Sin defectos.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="58" customHeight="1" s="45">
-      <c r="A15" s="75" t="inlineStr">
-        <is>
-          <t>UNIT-B08</t>
-        </is>
-      </c>
-      <c r="B15" s="76" t="inlineStr">
-        <is>
-          <t>Validación de nombre: caso corto</t>
-        </is>
-      </c>
-      <c r="C15" s="76" t="inlineStr">
-        <is>
-          <t>Función validate_name importada; sin BD ni servidor.</t>
-        </is>
-      </c>
-      <c r="D15" s="76" t="inlineStr">
-        <is>
-          <t>nombre="A"</t>
-        </is>
-      </c>
-      <c r="E15" s="76" t="inlineStr">
-        <is>
-          <t>1. Llamar validate_name(nombre). / 2. Capturar el valor booleano.</t>
-        </is>
-      </c>
-      <c r="F15" s="76" t="inlineStr">
-        <is>
-          <t>Retorna False (1 carácter).</t>
-        </is>
-      </c>
-      <c r="G15" s="76" t="inlineStr">
-        <is>
-          <t>Aprobado: retornó False.</t>
-        </is>
-      </c>
-      <c r="H15" s="76" t="inlineStr">
-        <is>
-          <t>Caja Blanca (Valor límite / partición)</t>
-        </is>
-      </c>
-      <c r="I15" s="74" t="inlineStr">
-        <is>
-          <t>Exitoso</t>
-        </is>
-      </c>
-      <c r="J15" s="75" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="K15" s="76" t="inlineStr">
-        <is>
-          <t>pytest api\tests\unit\test_unit_10_basicas.py -v: 10 passed; test_08_nombre_corto</t>
-        </is>
-      </c>
-      <c r="L15" s="76" t="inlineStr">
-        <is>
-          <t>Sin defectos.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="58" customHeight="1" s="45">
-      <c r="A16" s="72" t="inlineStr">
-        <is>
-          <t>UNIT-B09</t>
-        </is>
-      </c>
-      <c r="B16" s="73" t="inlineStr">
-        <is>
-          <t>Validación de fecha y hora: caso válido</t>
-        </is>
-      </c>
-      <c r="C16" s="73" t="inlineStr">
-        <is>
-          <t>Función validate_date_time importada; sin BD ni servidor.</t>
-        </is>
-      </c>
-      <c r="D16" s="73" t="inlineStr">
-        <is>
-          <t>fecha="2026-11-02" / hora="09:00"</t>
-        </is>
-      </c>
-      <c r="E16" s="73" t="inlineStr">
-        <is>
-          <t>1. Llamar validate_date_time(fecha, hora). / 2. Capturar el valor booleano.</t>
-        </is>
-      </c>
-      <c r="F16" s="73" t="inlineStr">
-        <is>
-          <t>Retorna True.</t>
-        </is>
-      </c>
-      <c r="G16" s="73" t="inlineStr">
-        <is>
-          <t>Aprobado: retornó True.</t>
-        </is>
-      </c>
-      <c r="H16" s="73" t="inlineStr">
-        <is>
-          <t>Caja Blanca (Formato / partición)</t>
-        </is>
-      </c>
-      <c r="I16" s="74" t="inlineStr">
-        <is>
-          <t>Exitoso</t>
-        </is>
-      </c>
-      <c r="J16" s="72" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="K16" s="73" t="inlineStr">
-        <is>
-          <t>pytest api\tests\unit\test_unit_10_basicas.py -v: 10 passed; test_09_fecha_y_hora_validas</t>
-        </is>
-      </c>
-      <c r="L16" s="73" t="inlineStr">
-        <is>
-          <t>Sin defectos.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="58" customHeight="1" s="45">
-      <c r="A17" s="75" t="inlineStr">
-        <is>
-          <t>UNIT-B10</t>
-        </is>
-      </c>
-      <c r="B17" s="76" t="inlineStr">
-        <is>
-          <t>Validación de fecha y hora: caso inválido</t>
-        </is>
-      </c>
-      <c r="C17" s="76" t="inlineStr">
-        <is>
-          <t>Función validate_date_time importada; sin BD ni servidor.</t>
-        </is>
-      </c>
-      <c r="D17" s="76" t="inlineStr">
-        <is>
-          <t>fecha="2026-13-01" / hora="09:00"</t>
-        </is>
-      </c>
-      <c r="E17" s="76" t="inlineStr">
-        <is>
-          <t>1. Llamar validate_date_time(fecha, hora). / 2. Capturar el valor booleano.</t>
-        </is>
-      </c>
-      <c r="F17" s="76" t="inlineStr">
-        <is>
-          <t>Retorna False (mes 13 inexistente).</t>
-        </is>
-      </c>
-      <c r="G17" s="76" t="inlineStr">
-        <is>
-          <t>Aprobado: retornó False.</t>
-        </is>
-      </c>
-      <c r="H17" s="76" t="inlineStr">
-        <is>
-          <t>Caja Blanca (Valor inválido / formato)</t>
-        </is>
-      </c>
-      <c r="I17" s="74" t="inlineStr">
-        <is>
-          <t>Exitoso</t>
-        </is>
-      </c>
-      <c r="J17" s="75" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="K17" s="76" t="inlineStr">
-        <is>
-          <t>pytest api\tests\unit\test_unit_10_basicas.py -v: 10 passed; test_10_fecha_y_hora_invalidas</t>
-        </is>
-      </c>
-      <c r="L17" s="76" t="inlineStr">
-        <is>
-          <t>Sin defectos.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="34" customHeight="1" s="45">
-      <c r="A19" s="77" t="inlineStr">
-        <is>
-          <t>NOTA: estas 10 pruebas unitarias básicas son un anexo de la entrega del aprendiz. No reemplazan los casos UNIT-01 a UNIT-05 del plan SENA ni modifican el resumen general de 12 casos.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A7:L17"/>
-  <mergeCells count="6">
-    <mergeCell ref="C3:F3"/>
-    <mergeCell ref="A19:L19"/>
-    <mergeCell ref="I3:L3"/>
-    <mergeCell ref="A1:L1"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="G3:H3"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>